<commit_message>
Fix translation leftovers and misaligned Exp3 tables
- Exp3 comparison tables: quote the R1-R4 hypothesis label so that every
  row has the same columns as the header again.
- Translate the remaining Italian labels in pilot_references.csv,
  supplementary_evidence_index.csv, tables.xlsx and two v4 CSVs.
- Rename the workbook theme of matrix.xlsx and tables.xlsx.
- experiments/README.md: list source_result among the unchanged raw columns.
- MANIFEST.csv: updated hashes of the corrected files.
</commit_message>
<xml_diff>
--- a/experiments/tables.xlsx
+++ b/experiments/tables.xlsx
@@ -627,9 +627,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="ChatGPT">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -679,7 +679,7 @@
         <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="ChatGPT">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="D42" s="12" t="inlineStr">
         <is>
-          <t>Invii blocked</t>
+          <t>Blocked sends</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
@@ -18415,7 +18415,7 @@
     <row r="23" ht="32" customHeight="1" s="25">
       <c r="C23" s="36" t="inlineStr">
         <is>
-          <t>v5: coverage input 14/29. Catalogo storico: 29 ID, Llama 3.2 3B e Qwen 2.5 7B, T=0,2 e 0,7.</t>
+          <t>v5: input coverage 14/29. Historical catalogue: 29 IDs, Llama 3.2 3B and Qwen 2.5 7B, T=0.2 and 0.7.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Point the workbook sources to the files in this package
- tables.xlsx, Method sheet: each source S01-S26 now names the package file
  that holds its data; the SHA-256 column is labelled as the hash of the
  original source file, with a note that those files are not included.
- MANIFEST.csv: updated hash of tables.xlsx.
</commit_message>
<xml_diff>
--- a/experiments/tables.xlsx
+++ b/experiments/tables.xlsx
@@ -18224,7 +18224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N64"/>
+  <dimension ref="B2:N67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" style="25" min="1" max="1"/>
@@ -18498,7 +18498,7 @@
     <row r="37">
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Sources included in the package</t>
+          <t>Sources of the tables</t>
         </is>
       </c>
     </row>
@@ -18510,12 +18510,12 @@
       </c>
       <c r="C39" s="35" t="inlineStr">
         <is>
-          <t>Description and attachment</t>
+          <t>Description and data in this package</t>
         </is>
       </c>
       <c r="D39" s="35" t="inlineStr">
         <is>
-          <t>SHA-256</t>
+          <t>SHA-256 of the original source file</t>
         </is>
       </c>
     </row>
@@ -18527,7 +18527,7 @@
       </c>
       <c r="C40" s="36" t="inlineStr">
         <is>
-          <t>Standard 0.2 (sources/S01-exp1_runs.csv)</t>
+          <t>Standard 0.2 (Exp1/per_run_data/exp1_runs.csv)</t>
         </is>
       </c>
       <c r="D40" s="36" t="inlineStr">
@@ -18544,7 +18544,7 @@
       </c>
       <c r="C41" s="36" t="inlineStr">
         <is>
-          <t>Seed replication 0.2 (sources/S02-exp1_runs.csv)</t>
+          <t>Seed replication 0.2 (Exp1/per_run_data/other_campaigns/seed_replication.csv)</t>
         </is>
       </c>
       <c r="D41" s="36" t="inlineStr">
@@ -18561,7 +18561,7 @@
       </c>
       <c r="C42" s="36" t="inlineStr">
         <is>
-          <t>Standard Qwen 0.7 (sources/S03-exp1_runs.csv)</t>
+          <t>Standard Qwen 0.7 (Exp1/per_run_data/other_campaigns/qwen_temperature07.csv)</t>
         </is>
       </c>
       <c r="D42" s="36" t="inlineStr">
@@ -18578,7 +18578,7 @@
       </c>
       <c r="C43" s="36" t="inlineStr">
         <is>
-          <t>JSON 0.2 (sources/S04-exp1_runs.csv)</t>
+          <t>JSON 0.2 (Exp1/per_run_data/other_campaigns/json_temperature02.csv)</t>
         </is>
       </c>
       <c r="D43" s="36" t="inlineStr">
@@ -18595,7 +18595,7 @@
       </c>
       <c r="C44" s="36" t="inlineStr">
         <is>
-          <t>JSON 0.7 (sources/S05-exp1_runs.csv)</t>
+          <t>JSON 0.7 (Exp1/per_run_data/other_campaigns/json_temperature07.csv)</t>
         </is>
       </c>
       <c r="D44" s="36" t="inlineStr">
@@ -18612,7 +18612,7 @@
       </c>
       <c r="C45" s="36" t="inlineStr">
         <is>
-          <t>Historical chain closure (sources/S06-chain-closure.json)</t>
+          <t>Historical chain closure (Exp1/chain_closure.json)</t>
         </is>
       </c>
       <c r="D45" s="36" t="inlineStr">
@@ -18629,7 +18629,7 @@
       </c>
       <c r="C46" s="36" t="inlineStr">
         <is>
-          <t>Historical catalogue (sources/S07-exp2_decisions.csv)</t>
+          <t>Historical catalogue (Exp2/historical_catalogue/exp2_results_29_scenarios.csv)</t>
         </is>
       </c>
       <c r="D46" s="36" t="inlineStr">
@@ -18646,7 +18646,7 @@
       </c>
       <c r="C47" s="36" t="inlineStr">
         <is>
-          <t>Benign control (sources/S08-exp2_decisions.csv)</t>
+          <t>Benign control (Exp2/benign_controls/benign_llama32_temperature02.csv)</t>
         </is>
       </c>
       <c r="D47" s="36" t="inlineStr">
@@ -18663,7 +18663,7 @@
       </c>
       <c r="C48" s="36" t="inlineStr">
         <is>
-          <t>v5, validation (24 texts) (sources/S10-decisions.csv)</t>
+          <t>v5, validation (24 texts) (Exp2/semantic_classification_v5/per_query_results.csv)</t>
         </is>
       </c>
       <c r="D48" s="36" t="inlineStr">
@@ -18680,7 +18680,7 @@
       </c>
       <c r="C49" s="36" t="inlineStr">
         <is>
-          <t>v5, development (sources/S11-decisions.csv)</t>
+          <t>v5, development (Exp2/semantic_classification_v5/per_query_results.csv)</t>
         </is>
       </c>
       <c r="D49" s="36" t="inlineStr">
@@ -18697,7 +18697,7 @@
       </c>
       <c r="C50" s="36" t="inlineStr">
         <is>
-          <t>v5, MCP captures (sources/S12-decisions.csv)</t>
+          <t>v5, MCP captures (Exp2/semantic_classification_v5/per_query_results.csv)</t>
         </is>
       </c>
       <c r="D50" s="36" t="inlineStr">
@@ -18714,7 +18714,7 @@
       </c>
       <c r="C51" s="36" t="inlineStr">
         <is>
-          <t>v5, static artifacts (sources/S13-decisions.csv)</t>
+          <t>v5, static artifacts (Exp2/semantic_classification_v5/per_query_results.csv)</t>
         </is>
       </c>
       <c r="D51" s="36" t="inlineStr">
@@ -18731,7 +18731,7 @@
       </c>
       <c r="C52" s="36" t="inlineStr">
         <is>
-          <t>v5, files and SQLite (sources/S14-decisions.csv)</t>
+          <t>v5, files and SQLite (Exp2/semantic_classification_v5/per_query_results.csv)</t>
         </is>
       </c>
       <c r="D52" s="36" t="inlineStr">
@@ -18748,7 +18748,7 @@
       </c>
       <c r="C53" s="36" t="inlineStr">
         <is>
-          <t>v5 coverage of the 29 IDs (sources/S15-coverage.json)</t>
+          <t>v5 coverage of the 29 IDs (Exp2/coverage_29_ids/coverage.csv)</t>
         </is>
       </c>
       <c r="D53" s="36" t="inlineStr">
@@ -18765,7 +18765,7 @@
       </c>
       <c r="C54" s="36" t="inlineStr">
         <is>
-          <t>STDIO comparison of MCTS and probes (sources/S16-exp3_compare.csv)</t>
+          <t>STDIO comparison of MCTS and probes (Exp3/comparison_14_targets/exp3_target_comparison.csv)</t>
         </is>
       </c>
       <c r="D54" s="36" t="inlineStr">
@@ -18782,7 +18782,7 @@
       </c>
       <c r="C55" s="36" t="inlineStr">
         <is>
-          <t>Cisco and Shield scans (sources/S17-results.csv)</t>
+          <t>Cisco and Shield scans (Exp3/comparison_14_targets/additional_scanners.csv)</t>
         </is>
       </c>
       <c r="D55" s="36" t="inlineStr">
@@ -18799,7 +18799,7 @@
       </c>
       <c r="C56" s="36" t="inlineStr">
         <is>
-          <t>Effects verified by the probes (sources/S18-exp3_effects.csv)</t>
+          <t>Effects verified by the probes (Exp3/probes_and_effects/probe_results.csv)</t>
         </is>
       </c>
       <c r="D56" s="36" t="inlineStr">
@@ -18816,7 +18816,7 @@
       </c>
       <c r="C57" s="36" t="inlineStr">
         <is>
-          <t>Five SSRF configurations (sources/S19-results.csv)</t>
+          <t>Five SSRF configurations (Exp3/ssrf_configurations/ssrf_results.csv)</t>
         </is>
       </c>
       <c r="D57" s="36" t="inlineStr">
@@ -18833,7 +18833,7 @@
       </c>
       <c r="C58" s="36" t="inlineStr">
         <is>
-          <t>P2 diagnostic checks (sources/S20-results.csv)</t>
+          <t>P2 diagnostic checks (Exp3/scanner_diagnostics/per_scan_results.csv)</t>
         </is>
       </c>
       <c r="D58" s="36" t="inlineStr">
@@ -18850,7 +18850,7 @@
       </c>
       <c r="C59" s="36" t="inlineStr">
         <is>
-          <t>Historical catalogue, llama3.2:3b, temperature 0.7 (sources/S21-exp2_decisions.csv)</t>
+          <t>Historical catalogue, llama3.2:3b, temperature 0.7 (Exp2/historical_catalogue/llama32_temperature07.csv)</t>
         </is>
       </c>
       <c r="D59" s="36" t="inlineStr">
@@ -18867,7 +18867,7 @@
       </c>
       <c r="C60" s="36" t="inlineStr">
         <is>
-          <t>Historical benign controls, llama3.2:3b, temperature 0.7 (sources/S22-exp2_decisions.csv)</t>
+          <t>Historical benign controls, llama3.2:3b, temperature 0.7 (Exp2/benign_controls/benign_llama32_temperature07.csv)</t>
         </is>
       </c>
       <c r="D60" s="36" t="inlineStr">
@@ -18884,7 +18884,7 @@
       </c>
       <c r="C61" s="36" t="inlineStr">
         <is>
-          <t>Historical catalogue, qwen2.5:7b, temperature 0.2 (sources/S23-exp2_decisions.csv)</t>
+          <t>Historical catalogue, qwen2.5:7b, temperature 0.2 (Exp2/historical_catalogue/qwen25_temperature02.csv)</t>
         </is>
       </c>
       <c r="D61" s="36" t="inlineStr">
@@ -18901,7 +18901,7 @@
       </c>
       <c r="C62" s="36" t="inlineStr">
         <is>
-          <t>Historical benign controls, qwen2.5:7b, temperature 0.2 (sources/S24-exp2_decisions.csv)</t>
+          <t>Historical benign controls, qwen2.5:7b, temperature 0.2 (Exp2/benign_controls/benign_qwen25_temperature02.csv)</t>
         </is>
       </c>
       <c r="D62" s="36" t="inlineStr">
@@ -18918,7 +18918,7 @@
       </c>
       <c r="C63" s="36" t="inlineStr">
         <is>
-          <t>Historical catalogue, qwen2.5:7b, temperature 0.7 (sources/S25-exp2_decisions.csv)</t>
+          <t>Historical catalogue, qwen2.5:7b, temperature 0.7 (Exp2/historical_catalogue/qwen25_temperature07.csv)</t>
         </is>
       </c>
       <c r="D63" s="36" t="inlineStr">
@@ -18935,12 +18935,26 @@
       </c>
       <c r="C64" s="36" t="inlineStr">
         <is>
-          <t>Historical benign controls, qwen2.5:7b, temperature 0.7 (sources/S26-exp2_decisions.csv)</t>
+          <t>Historical benign controls, qwen2.5:7b, temperature 0.7 (Exp2/benign_controls/benign_qwen25_temperature07.csv)</t>
         </is>
       </c>
       <c r="D64" s="36" t="inlineStr">
         <is>
           <t>0f724c3c5584b1875e0c12abfb156cd41a15600a21757603f600c7757fa64796</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="24" t="inlineStr">
+        <is>
+          <t>The SHA-256 values identify the original source files from which these tables were built; apart from S06, those files are not part of this package.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="24" t="inlineStr">
+        <is>
+          <t>The data used here are in the files listed in the description column, also indexed in evidence/result_sources.csv.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Repair the Excel tables in tables.xlsx
- The 15 Excel tables now use the English header names and English table
  names; Italian column names left in the table definitions made Excel
  report the workbook as damaged.
- Restore the cached results of the 546 formulas, lost when the
  translated workbook was saved; the formulas are unchanged.
- MANIFEST.csv: updated hash of tables.xlsx.
</commit_message>
<xml_diff>
--- a/experiments/tables.xlsx
+++ b/experiments/tables.xlsx
@@ -351,29 +351,29 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T01_exp1_campagne" displayName="T01_exp1_campagne" ref="B8:N13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="T01_exp1_campaigns" displayName="T01_exp1_campaigns" ref="B8:N13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="B8:N13"/>
   <tableColumns count="13">
-    <tableColumn id="1" name="Campagna"/>
+    <tableColumn id="1" name="Campaign"/>
     <tableColumn id="2" name="T"/>
     <tableColumn id="3" name="N"/>
     <tableColumn id="4" name="D"/>
     <tableColumn id="5" name="A"/>
     <tableColumn id="6" name="E"/>
     <tableColumn id="7" name="U"/>
-    <tableColumn id="8" name="Errori"/>
+    <tableColumn id="8" name="Errors"/>
     <tableColumn id="9" name="D %"/>
     <tableColumn id="10" name="A %"/>
     <tableColumn id="11" name="E %"/>
     <tableColumn id="12" name="U %"/>
-    <tableColumn id="13" name="Fonte"/>
+    <tableColumn id="13" name="Source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T08_exp2_benigni" displayName="T08_exp2_benigni" ref="B197:J201" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="T08_exp2_benign" displayName="T08_exp2_benign" ref="B197:J201" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="B197:J201"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Scenario"/>
@@ -381,56 +381,56 @@
     <tableColumn id="3" name="Exfiltrate"/>
     <tableColumn id="4" name="Ignore"/>
     <tableColumn id="5" name="Unknown"/>
-    <tableColumn id="6" name="Errori"/>
+    <tableColumn id="6" name="Errors"/>
     <tableColumn id="7" name="T"/>
-    <tableColumn id="8" name="Modello"/>
-    <tableColumn id="9" name="Fonte"/>
+    <tableColumn id="8" name="Model"/>
+    <tableColumn id="9" name="Source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="T09_exp2_copertura" displayName="T09_exp2_copertura" ref="B208:F237" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="T09_exp2_coverage" displayName="T09_exp2_coverage" ref="B208:F237" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="B208:F237"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
-    <tableColumn id="2" name="Copertura"/>
-    <tableColumn id="3" name="Superficie"/>
-    <tableColumn id="4" name="Alias di"/>
-    <tableColumn id="5" name="Fonte"/>
+    <tableColumn id="2" name="Coverage"/>
+    <tableColumn id="3" name="Surface"/>
+    <tableColumn id="4" name="Alias of"/>
+    <tableColumn id="5" name="Source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="T10_exp3_target" displayName="T10_exp3_target" ref="B8:I22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="T10_exp3_targets" displayName="T10_exp3_targets" ref="B8:I22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="B8:I22"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Target"/>
-    <tableColumn id="2" name="Ipotesi iniziale"/>
-    <tableColumn id="3" name="MCTS generico"/>
-    <tableColumn id="4" name="Sonde P2"/>
+    <tableColumn id="2" name="Initial hypothesis"/>
+    <tableColumn id="3" name="MCTS generic"/>
+    <tableColumn id="4" name="P2 probes"/>
     <tableColumn id="5" name="Cisco YARA"/>
     <tableColumn id="6" name="Shield"/>
-    <tableColumn id="7" name="Sonde: effetto"/>
-    <tableColumn id="8" name="Fonti"/>
+    <tableColumn id="7" name="Probes: effect"/>
+    <tableColumn id="8" name="Sources"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="T11_exp3_sonde" displayName="T11_exp3_sonde" ref="B31:G37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="T11_exp3_probes" displayName="T11_exp3_probes" ref="B31:G37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="B31:G37"/>
   <tableColumns count="6">
     <tableColumn id="1" name="Target"/>
-    <tableColumn id="2" name="Sonda"/>
-    <tableColumn id="3" name="Profilo"/>
-    <tableColumn id="4" name="Esito"/>
-    <tableColumn id="5" name="Evidenza o limite"/>
-    <tableColumn id="6" name="Fonte"/>
+    <tableColumn id="2" name="Probe"/>
+    <tableColumn id="3" name="Profile"/>
+    <tableColumn id="4" name="Outcome"/>
+    <tableColumn id="5" name="Evidence or limit"/>
+    <tableColumn id="6" name="Source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -440,32 +440,32 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="T12_exp3_ssrf" displayName="T12_exp3_ssrf" ref="B44:I49" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="B44:I49"/>
   <tableColumns count="8">
-    <tableColumn id="1" name="Pacchetto"/>
-    <tableColumn id="2" name="Versione"/>
-    <tableColumn id="3" name="Esito P6"/>
-    <tableColumn id="4" name="Tentativi"/>
-    <tableColumn id="5" name="Respinti policy"/>
-    <tableColumn id="6" name="Sweep completo"/>
+    <tableColumn id="1" name="Package"/>
+    <tableColumn id="2" name="Version"/>
+    <tableColumn id="3" name="P6 outcome"/>
+    <tableColumn id="4" name="Attempts"/>
+    <tableColumn id="5" name="Policy rejections"/>
+    <tableColumn id="6" name="Complete sweep"/>
     <tableColumn id="7" name="MCTS SSRF"/>
-    <tableColumn id="8" name="Fonte"/>
+    <tableColumn id="8" name="Source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="T13_exp3_diagnostica" displayName="T13_exp3_diagnostica" ref="B58:J61" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="T13_exp3_diagnostics" displayName="T13_exp3_diagnostics" ref="B58:J61" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="B58:J61"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Scanner"/>
-    <tableColumn id="2" name="Malevoli"/>
-    <tableColumn id="3" name="Benigni"/>
+    <tableColumn id="2" name="Malicious"/>
+    <tableColumn id="3" name="Benign"/>
     <tableColumn id="4" name="TP"/>
     <tableColumn id="5" name="TN"/>
     <tableColumn id="6" name="FP"/>
     <tableColumn id="7" name="FN"/>
-    <tableColumn id="8" name="Errori"/>
-    <tableColumn id="9" name="Fonte"/>
+    <tableColumn id="8" name="Errors"/>
+    <tableColumn id="9" name="Source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -476,8 +476,8 @@
   <autoFilter ref="B22:L34"/>
   <tableColumns count="11">
     <tableColumn id="1" name="T"/>
-    <tableColumn id="2" name="Modello"/>
-    <tableColumn id="3" name="Profilo"/>
+    <tableColumn id="2" name="Model"/>
+    <tableColumn id="3" name="Profile"/>
     <tableColumn id="4" name="N"/>
     <tableColumn id="5" name="D"/>
     <tableColumn id="6" name="A"/>
@@ -485,22 +485,22 @@
     <tableColumn id="8" name="U"/>
     <tableColumn id="9" name="E %"/>
     <tableColumn id="10" name="U %"/>
-    <tableColumn id="11" name="Fonte"/>
+    <tableColumn id="11" name="Source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T03_exp1_difese" displayName="T03_exp1_difese" ref="B42:I44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T03_exp1_defences" displayName="T03_exp1_defences" ref="B42:I44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="B42:I44"/>
   <tableColumns count="8">
     <tableColumn id="1" name="T"/>
     <tableColumn id="2" name="N"/>
-    <tableColumn id="3" name="Invii bloccati"/>
-    <tableColumn id="4" name="Run con lettura"/>
-    <tableColumn id="5" name="Run con redazione"/>
-    <tableColumn id="6" name="Run con token visibile"/>
+    <tableColumn id="3" name="Blocked sends"/>
+    <tableColumn id="4" name="Runs with a read"/>
+    <tableColumn id="5" name="Runs with redaction"/>
+    <tableColumn id="6" name="Runs with a visible token"/>
     <tableColumn id="7" name="A"/>
     <tableColumn id="8" name="E"/>
   </tableColumns>
@@ -509,35 +509,35 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T04_exp1_catene" displayName="T04_exp1_catene" ref="B52:L53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T04_exp1_chains" displayName="T04_exp1_chains" ref="B52:L53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="B52:L53"/>
   <tableColumns count="11">
-    <tableColumn id="1" name="Pianificate"/>
-    <tableColumn id="2" name="Registrate"/>
+    <tableColumn id="1" name="Planned"/>
+    <tableColumn id="2" name="Recorded"/>
     <tableColumn id="3" name="Timeout"/>
-    <tableColumn id="4" name="Perse"/>
-    <tableColumn id="5" name="Utilizzabili"/>
+    <tableColumn id="4" name="Lost"/>
+    <tableColumn id="5" name="Usable"/>
     <tableColumn id="6" name="D"/>
     <tableColumn id="7" name="A"/>
     <tableColumn id="8" name="E"/>
     <tableColumn id="9" name="U"/>
     <tableColumn id="10" name="U %"/>
-    <tableColumn id="11" name="Fonte"/>
+    <tableColumn id="11" name="Source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="T05_exp1_celle" displayName="T05_exp1_celle" ref="B62:Q186" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="T05_exp1_cells" displayName="T05_exp1_cells" ref="B62:Q186" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="B62:Q186"/>
   <tableColumns count="16">
-    <tableColumn id="1" name="Campagna"/>
+    <tableColumn id="1" name="Campaign"/>
     <tableColumn id="2" name="T"/>
-    <tableColumn id="3" name="Modello"/>
+    <tableColumn id="3" name="Model"/>
     <tableColumn id="4" name="Scenario"/>
     <tableColumn id="5" name="Task"/>
-    <tableColumn id="6" name="Profilo"/>
+    <tableColumn id="6" name="Profile"/>
     <tableColumn id="7" name="N"/>
     <tableColumn id="8" name="D"/>
     <tableColumn id="9" name="A"/>
@@ -547,55 +547,55 @@
     <tableColumn id="13" name="A %"/>
     <tableColumn id="14" name="E %"/>
     <tableColumn id="15" name="U %"/>
-    <tableColumn id="16" name="Fonte"/>
+    <tableColumn id="16" name="Source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="T06_exp2_classificazione" displayName="T06_exp2_classificazione" ref="B8:M13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="T06_exp2_classification" displayName="T06_exp2_classification" ref="B8:M13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="B8:M13"/>
   <tableColumns count="12">
-    <tableColumn id="1" name="Campione"/>
-    <tableColumn id="2" name="Testi"/>
+    <tableColumn id="1" name="Sample"/>
+    <tableColumn id="2" name="Texts"/>
     <tableColumn id="3" name="Query"/>
     <tableColumn id="4" name="TP"/>
     <tableColumn id="5" name="TN"/>
     <tableColumn id="6" name="FP"/>
     <tableColumn id="7" name="FN"/>
     <tableColumn id="8" name="Unknown"/>
-    <tableColumn id="9" name="Corrette"/>
-    <tableColumn id="10" name="Corrette %"/>
-    <tableColumn id="11" name="Errori"/>
-    <tableColumn id="12" name="Fonte"/>
+    <tableColumn id="9" name="Correct"/>
+    <tableColumn id="10" name="Correct %"/>
+    <tableColumn id="11" name="Errors"/>
+    <tableColumn id="12" name="Source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="T14_exp2_modelli_temperature" displayName="T14_exp2_modelli_temperature" ref="B24:L28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="T14_exp2_models_temperatures" displayName="T14_exp2_models_temperatures" ref="B24:L28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="B24:L28"/>
   <tableColumns count="11">
-    <tableColumn id="1" name="Modello"/>
-    <tableColumn id="2" name="Temperatura"/>
+    <tableColumn id="1" name="Model"/>
+    <tableColumn id="2" name="Temperature"/>
     <tableColumn id="3" name="ID"/>
     <tableColumn id="4" name="Query"/>
     <tableColumn id="5" name="Exfiltrate"/>
     <tableColumn id="6" name="Ignore"/>
     <tableColumn id="7" name="Unknown"/>
-    <tableColumn id="8" name="Errori"/>
-    <tableColumn id="9" name="ID positivi"/>
-    <tableColumn id="10" name="Testi distinti"/>
-    <tableColumn id="11" name="Fonte"/>
+    <tableColumn id="8" name="Errors"/>
+    <tableColumn id="9" name="Positive IDs"/>
+    <tableColumn id="10" name="Distinct texts"/>
+    <tableColumn id="11" name="Source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T15_exp2_confronto_29_id" displayName="T15_exp2_confronto_29_id" ref="B35:F64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="T15_exp2_comparison_29_ids" displayName="T15_exp2_comparison_29_ids" ref="B35:F64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="B35:F64"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Scenario"/>
@@ -609,7 +609,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="T07_exp2_storico" displayName="T07_exp2_storico" ref="B73:J189" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="T07_exp2_historical" displayName="T07_exp2_historical" ref="B73:J189" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="B73:J189"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Scenario"/>
@@ -617,10 +617,10 @@
     <tableColumn id="3" name="Exfiltrate"/>
     <tableColumn id="4" name="Ignore"/>
     <tableColumn id="5" name="Unknown"/>
-    <tableColumn id="6" name="Errori"/>
+    <tableColumn id="6" name="Errors"/>
     <tableColumn id="7" name="T"/>
-    <tableColumn id="8" name="Modello"/>
-    <tableColumn id="9" name="Fonte"/>
+    <tableColumn id="8" name="Model"/>
+    <tableColumn id="9" name="Source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -824,7 +824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:Q186"/>
+  <dimension ref="A1:Q186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" style="25" min="1" max="1"/>
@@ -846,6 +846,7 @@
     <col width="8" customWidth="1" style="25" min="17" max="17"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="26" customHeight="1" s="25">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -875,6 +876,7 @@
       <c r="M4" s="3" t="n"/>
       <c r="N4" s="3" t="n"/>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
@@ -882,6 +884,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="34" customHeight="1" s="25">
       <c r="B8" s="11" t="inlineStr">
         <is>
@@ -978,19 +981,19 @@
       </c>
       <c r="J9" s="49">
         <f>E9/D9</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K9" s="49">
         <f>F9/D9</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L9" s="49">
         <f>G9/D9</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M9" s="49">
         <f>H9/D9</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="N9" s="29" t="inlineStr">
         <is>
@@ -1027,19 +1030,19 @@
       </c>
       <c r="J10" s="52">
         <f>E10/D10</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K10" s="52">
         <f>F10/D10</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L10" s="52">
         <f>G10/D10</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M10" s="52">
         <f>H10/D10</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="N10" s="30" t="inlineStr">
         <is>
@@ -1076,19 +1079,19 @@
       </c>
       <c r="J11" s="49">
         <f>E11/D11</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K11" s="49">
         <f>F11/D11</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L11" s="49">
         <f>G11/D11</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="M11" s="49">
         <f>H11/D11</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="N11" s="29" t="inlineStr">
         <is>
@@ -1125,19 +1128,19 @@
       </c>
       <c r="J12" s="52">
         <f>E12/D12</f>
-        <v/>
+        <v>0.125</v>
       </c>
       <c r="K12" s="52">
         <f>F12/D12</f>
-        <v/>
+        <v>0.05</v>
       </c>
       <c r="L12" s="52">
         <f>G12/D12</f>
-        <v/>
+        <v>0.03333333333333333</v>
       </c>
       <c r="M12" s="52">
         <f>H12/D12</f>
-        <v/>
+        <v>0.7583333333333333</v>
       </c>
       <c r="N12" s="30" t="inlineStr">
         <is>
@@ -1174,19 +1177,19 @@
       </c>
       <c r="J13" s="49">
         <f>E13/D13</f>
-        <v/>
+        <v>0.16666666666666666</v>
       </c>
       <c r="K13" s="49">
         <f>F13/D13</f>
-        <v/>
+        <v>0.09166666666666666</v>
       </c>
       <c r="L13" s="49">
         <f>G13/D13</f>
-        <v/>
+        <v>0.06666666666666667</v>
       </c>
       <c r="M13" s="49">
         <f>H13/D13</f>
-        <v/>
+        <v>0.7833333333333333</v>
       </c>
       <c r="N13" s="29" t="inlineStr">
         <is>
@@ -1194,6 +1197,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="19" customHeight="1" s="25">
       <c r="B15" s="24" t="inlineStr">
         <is>
@@ -1215,6 +1219,8 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
     <row r="20">
       <c r="B20" s="4" t="inlineStr">
         <is>
@@ -1222,6 +1228,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="34" customHeight="1" s="25">
       <c r="B22" s="11" t="inlineStr">
         <is>
@@ -1310,11 +1317,11 @@
       </c>
       <c r="J23" s="49">
         <f>H23/E23</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K23" s="49">
         <f>I23/E23</f>
-        <v/>
+        <v>0.65</v>
       </c>
       <c r="L23" s="29" t="inlineStr">
         <is>
@@ -1353,11 +1360,11 @@
       </c>
       <c r="J24" s="52">
         <f>H24/E24</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K24" s="52">
         <f>I24/E24</f>
-        <v/>
+        <v>0.7</v>
       </c>
       <c r="L24" s="30" t="inlineStr">
         <is>
@@ -1396,11 +1403,11 @@
       </c>
       <c r="J25" s="49">
         <f>H25/E25</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K25" s="49">
         <f>I25/E25</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="L25" s="29" t="inlineStr">
         <is>
@@ -1439,11 +1446,11 @@
       </c>
       <c r="J26" s="52">
         <f>H26/E26</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K26" s="52">
         <f>I26/E26</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="L26" s="30" t="inlineStr">
         <is>
@@ -1482,11 +1489,11 @@
       </c>
       <c r="J27" s="49">
         <f>H27/E27</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K27" s="49">
         <f>I27/E27</f>
-        <v/>
+        <v>0.5</v>
       </c>
       <c r="L27" s="29" t="inlineStr">
         <is>
@@ -1525,11 +1532,11 @@
       </c>
       <c r="J28" s="52">
         <f>H28/E28</f>
-        <v/>
+        <v>0.2</v>
       </c>
       <c r="K28" s="52">
         <f>I28/E28</f>
-        <v/>
+        <v>0.7</v>
       </c>
       <c r="L28" s="30" t="inlineStr">
         <is>
@@ -1568,11 +1575,11 @@
       </c>
       <c r="J29" s="49">
         <f>H29/E29</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K29" s="49">
         <f>I29/E29</f>
-        <v/>
+        <v>0.7</v>
       </c>
       <c r="L29" s="29" t="inlineStr">
         <is>
@@ -1611,11 +1618,11 @@
       </c>
       <c r="J30" s="52">
         <f>H30/E30</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K30" s="52">
         <f>I30/E30</f>
-        <v/>
+        <v>0.9</v>
       </c>
       <c r="L30" s="30" t="inlineStr">
         <is>
@@ -1654,11 +1661,11 @@
       </c>
       <c r="J31" s="49">
         <f>H31/E31</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K31" s="49">
         <f>I31/E31</f>
-        <v/>
+        <v>0.95</v>
       </c>
       <c r="L31" s="29" t="inlineStr">
         <is>
@@ -1697,11 +1704,11 @@
       </c>
       <c r="J32" s="52">
         <f>H32/E32</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K32" s="52">
         <f>I32/E32</f>
-        <v/>
+        <v>0.95</v>
       </c>
       <c r="L32" s="30" t="inlineStr">
         <is>
@@ -1740,11 +1747,11 @@
       </c>
       <c r="J33" s="49">
         <f>H33/E33</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K33" s="49">
         <f>I33/E33</f>
-        <v/>
+        <v>0.65</v>
       </c>
       <c r="L33" s="29" t="inlineStr">
         <is>
@@ -1783,11 +1790,11 @@
       </c>
       <c r="J34" s="52">
         <f>H34/E34</f>
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="K34" s="52">
         <f>I34/E34</f>
-        <v/>
+        <v>0.55</v>
       </c>
       <c r="L34" s="30" t="inlineStr">
         <is>
@@ -1795,6 +1802,7 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
     <row r="36" ht="19" customHeight="1" s="25">
       <c r="B36" s="24" t="inlineStr">
         <is>
@@ -1809,6 +1817,8 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
+    <row r="39"/>
     <row r="40">
       <c r="B40" s="4" t="inlineStr">
         <is>
@@ -1816,6 +1826,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42" ht="34" customHeight="1" s="25">
       <c r="B42" s="11" t="inlineStr">
         <is>
@@ -1910,6 +1921,7 @@
         <v>0</v>
       </c>
     </row>
+    <row r="45"/>
     <row r="46" ht="19" customHeight="1" s="25">
       <c r="B46" s="24" t="inlineStr">
         <is>
@@ -1924,6 +1936,8 @@
         </is>
       </c>
     </row>
+    <row r="48"/>
+    <row r="49"/>
     <row r="50">
       <c r="B50" s="4" t="inlineStr">
         <is>
@@ -1931,6 +1945,7 @@
         </is>
       </c>
     </row>
+    <row r="51"/>
     <row r="52" ht="34" customHeight="1" s="25">
       <c r="B52" s="11" t="inlineStr">
         <is>
@@ -2018,7 +2033,7 @@
       </c>
       <c r="K53" s="49">
         <f>J53/F53</f>
-        <v/>
+        <v>0.4518201284796574</v>
       </c>
       <c r="L53" s="29" t="inlineStr">
         <is>
@@ -2026,6 +2041,7 @@
         </is>
       </c>
     </row>
+    <row r="54"/>
     <row r="55" ht="19" customHeight="1" s="25">
       <c r="B55" s="24" t="inlineStr">
         <is>
@@ -2047,6 +2063,8 @@
         </is>
       </c>
     </row>
+    <row r="58"/>
+    <row r="59"/>
     <row r="60">
       <c r="B60" s="4" t="inlineStr">
         <is>
@@ -2054,6 +2072,7 @@
         </is>
       </c>
     </row>
+    <row r="61"/>
     <row r="62" ht="34" customHeight="1" s="25">
       <c r="B62" s="11" t="inlineStr">
         <is>
@@ -2182,19 +2201,19 @@
       </c>
       <c r="M63" s="49">
         <f>I63/H63</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N63" s="49">
         <f>J63/H63</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O63" s="49">
         <f>K63/H63</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P63" s="49">
         <f>L63/H63</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q63" s="29" t="inlineStr">
         <is>
@@ -2248,19 +2267,19 @@
       </c>
       <c r="M64" s="52">
         <f>I64/H64</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N64" s="52">
         <f>J64/H64</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O64" s="52">
         <f>K64/H64</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P64" s="52">
         <f>L64/H64</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q64" s="30" t="inlineStr">
         <is>
@@ -2314,19 +2333,19 @@
       </c>
       <c r="M65" s="49">
         <f>I65/H65</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N65" s="49">
         <f>J65/H65</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O65" s="49">
         <f>K65/H65</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P65" s="49">
         <f>L65/H65</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q65" s="29" t="inlineStr">
         <is>
@@ -2380,19 +2399,19 @@
       </c>
       <c r="M66" s="52">
         <f>I66/H66</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N66" s="52">
         <f>J66/H66</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O66" s="52">
         <f>K66/H66</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P66" s="52">
         <f>L66/H66</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q66" s="30" t="inlineStr">
         <is>
@@ -2446,19 +2465,19 @@
       </c>
       <c r="M67" s="49">
         <f>I67/H67</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N67" s="49">
         <f>J67/H67</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O67" s="49">
         <f>K67/H67</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P67" s="49">
         <f>L67/H67</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q67" s="29" t="inlineStr">
         <is>
@@ -2512,19 +2531,19 @@
       </c>
       <c r="M68" s="52">
         <f>I68/H68</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N68" s="52">
         <f>J68/H68</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O68" s="52">
         <f>K68/H68</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P68" s="52">
         <f>L68/H68</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q68" s="30" t="inlineStr">
         <is>
@@ -2578,19 +2597,19 @@
       </c>
       <c r="M69" s="49">
         <f>I69/H69</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N69" s="49">
         <f>J69/H69</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O69" s="49">
         <f>K69/H69</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P69" s="49">
         <f>L69/H69</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q69" s="29" t="inlineStr">
         <is>
@@ -2644,19 +2663,19 @@
       </c>
       <c r="M70" s="52">
         <f>I70/H70</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N70" s="52">
         <f>J70/H70</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O70" s="52">
         <f>K70/H70</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P70" s="52">
         <f>L70/H70</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q70" s="30" t="inlineStr">
         <is>
@@ -2710,19 +2729,19 @@
       </c>
       <c r="M71" s="49">
         <f>I71/H71</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N71" s="49">
         <f>J71/H71</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O71" s="49">
         <f>K71/H71</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P71" s="49">
         <f>L71/H71</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q71" s="29" t="inlineStr">
         <is>
@@ -2776,19 +2795,19 @@
       </c>
       <c r="M72" s="52">
         <f>I72/H72</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N72" s="52">
         <f>J72/H72</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O72" s="52">
         <f>K72/H72</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P72" s="52">
         <f>L72/H72</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q72" s="30" t="inlineStr">
         <is>
@@ -2842,19 +2861,19 @@
       </c>
       <c r="M73" s="49">
         <f>I73/H73</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N73" s="49">
         <f>J73/H73</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O73" s="49">
         <f>K73/H73</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P73" s="49">
         <f>L73/H73</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q73" s="29" t="inlineStr">
         <is>
@@ -2908,19 +2927,19 @@
       </c>
       <c r="M74" s="52">
         <f>I74/H74</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N74" s="52">
         <f>J74/H74</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O74" s="52">
         <f>K74/H74</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P74" s="52">
         <f>L74/H74</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q74" s="30" t="inlineStr">
         <is>
@@ -2974,19 +2993,19 @@
       </c>
       <c r="M75" s="49">
         <f>I75/H75</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N75" s="49">
         <f>J75/H75</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O75" s="49">
         <f>K75/H75</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P75" s="49">
         <f>L75/H75</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q75" s="29" t="inlineStr">
         <is>
@@ -3040,19 +3059,19 @@
       </c>
       <c r="M76" s="52">
         <f>I76/H76</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N76" s="52">
         <f>J76/H76</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O76" s="52">
         <f>K76/H76</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P76" s="52">
         <f>L76/H76</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q76" s="30" t="inlineStr">
         <is>
@@ -3106,19 +3125,19 @@
       </c>
       <c r="M77" s="49">
         <f>I77/H77</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N77" s="49">
         <f>J77/H77</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O77" s="49">
         <f>K77/H77</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P77" s="49">
         <f>L77/H77</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q77" s="29" t="inlineStr">
         <is>
@@ -3172,19 +3191,19 @@
       </c>
       <c r="M78" s="52">
         <f>I78/H78</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N78" s="52">
         <f>J78/H78</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O78" s="52">
         <f>K78/H78</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P78" s="52">
         <f>L78/H78</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q78" s="30" t="inlineStr">
         <is>
@@ -3238,19 +3257,19 @@
       </c>
       <c r="M79" s="49">
         <f>I79/H79</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N79" s="49">
         <f>J79/H79</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O79" s="49">
         <f>K79/H79</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P79" s="49">
         <f>L79/H79</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q79" s="29" t="inlineStr">
         <is>
@@ -3304,19 +3323,19 @@
       </c>
       <c r="M80" s="52">
         <f>I80/H80</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N80" s="52">
         <f>J80/H80</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O80" s="52">
         <f>K80/H80</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P80" s="52">
         <f>L80/H80</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q80" s="30" t="inlineStr">
         <is>
@@ -3370,19 +3389,19 @@
       </c>
       <c r="M81" s="49">
         <f>I81/H81</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N81" s="49">
         <f>J81/H81</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O81" s="49">
         <f>K81/H81</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P81" s="49">
         <f>L81/H81</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q81" s="29" t="inlineStr">
         <is>
@@ -3436,19 +3455,19 @@
       </c>
       <c r="M82" s="52">
         <f>I82/H82</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N82" s="52">
         <f>J82/H82</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O82" s="52">
         <f>K82/H82</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P82" s="52">
         <f>L82/H82</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q82" s="30" t="inlineStr">
         <is>
@@ -3502,19 +3521,19 @@
       </c>
       <c r="M83" s="49">
         <f>I83/H83</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N83" s="49">
         <f>J83/H83</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O83" s="49">
         <f>K83/H83</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P83" s="49">
         <f>L83/H83</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q83" s="29" t="inlineStr">
         <is>
@@ -3568,19 +3587,19 @@
       </c>
       <c r="M84" s="52">
         <f>I84/H84</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N84" s="52">
         <f>J84/H84</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O84" s="52">
         <f>K84/H84</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P84" s="52">
         <f>L84/H84</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q84" s="30" t="inlineStr">
         <is>
@@ -3634,19 +3653,19 @@
       </c>
       <c r="M85" s="49">
         <f>I85/H85</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N85" s="49">
         <f>J85/H85</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O85" s="49">
         <f>K85/H85</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P85" s="49">
         <f>L85/H85</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q85" s="29" t="inlineStr">
         <is>
@@ -3700,19 +3719,19 @@
       </c>
       <c r="M86" s="52">
         <f>I86/H86</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N86" s="52">
         <f>J86/H86</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O86" s="52">
         <f>K86/H86</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P86" s="52">
         <f>L86/H86</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q86" s="30" t="inlineStr">
         <is>
@@ -3766,19 +3785,19 @@
       </c>
       <c r="M87" s="49">
         <f>I87/H87</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N87" s="49">
         <f>J87/H87</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O87" s="49">
         <f>K87/H87</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P87" s="49">
         <f>L87/H87</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q87" s="29" t="inlineStr">
         <is>
@@ -3832,19 +3851,19 @@
       </c>
       <c r="M88" s="52">
         <f>I88/H88</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N88" s="52">
         <f>J88/H88</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O88" s="52">
         <f>K88/H88</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P88" s="52">
         <f>L88/H88</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q88" s="30" t="inlineStr">
         <is>
@@ -3898,19 +3917,19 @@
       </c>
       <c r="M89" s="49">
         <f>I89/H89</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N89" s="49">
         <f>J89/H89</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O89" s="49">
         <f>K89/H89</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P89" s="49">
         <f>L89/H89</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q89" s="29" t="inlineStr">
         <is>
@@ -3964,19 +3983,19 @@
       </c>
       <c r="M90" s="52">
         <f>I90/H90</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N90" s="52">
         <f>J90/H90</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O90" s="52">
         <f>K90/H90</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P90" s="52">
         <f>L90/H90</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q90" s="30" t="inlineStr">
         <is>
@@ -4030,19 +4049,19 @@
       </c>
       <c r="M91" s="49">
         <f>I91/H91</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N91" s="49">
         <f>J91/H91</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O91" s="49">
         <f>K91/H91</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P91" s="49">
         <f>L91/H91</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q91" s="29" t="inlineStr">
         <is>
@@ -4096,19 +4115,19 @@
       </c>
       <c r="M92" s="52">
         <f>I92/H92</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N92" s="52">
         <f>J92/H92</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O92" s="52">
         <f>K92/H92</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P92" s="52">
         <f>L92/H92</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q92" s="30" t="inlineStr">
         <is>
@@ -4162,19 +4181,19 @@
       </c>
       <c r="M93" s="49">
         <f>I93/H93</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N93" s="49">
         <f>J93/H93</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O93" s="49">
         <f>K93/H93</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P93" s="49">
         <f>L93/H93</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q93" s="29" t="inlineStr">
         <is>
@@ -4228,19 +4247,19 @@
       </c>
       <c r="M94" s="52">
         <f>I94/H94</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N94" s="52">
         <f>J94/H94</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O94" s="52">
         <f>K94/H94</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P94" s="52">
         <f>L94/H94</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q94" s="30" t="inlineStr">
         <is>
@@ -4294,19 +4313,19 @@
       </c>
       <c r="M95" s="49">
         <f>I95/H95</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N95" s="49">
         <f>J95/H95</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O95" s="49">
         <f>K95/H95</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P95" s="49">
         <f>L95/H95</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q95" s="29" t="inlineStr">
         <is>
@@ -4360,19 +4379,19 @@
       </c>
       <c r="M96" s="52">
         <f>I96/H96</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N96" s="52">
         <f>J96/H96</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O96" s="52">
         <f>K96/H96</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P96" s="52">
         <f>L96/H96</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q96" s="30" t="inlineStr">
         <is>
@@ -4426,19 +4445,19 @@
       </c>
       <c r="M97" s="49">
         <f>I97/H97</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N97" s="49">
         <f>J97/H97</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O97" s="49">
         <f>K97/H97</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P97" s="49">
         <f>L97/H97</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q97" s="29" t="inlineStr">
         <is>
@@ -4492,19 +4511,19 @@
       </c>
       <c r="M98" s="52">
         <f>I98/H98</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N98" s="52">
         <f>J98/H98</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O98" s="52">
         <f>K98/H98</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P98" s="52">
         <f>L98/H98</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q98" s="30" t="inlineStr">
         <is>
@@ -4558,19 +4577,19 @@
       </c>
       <c r="M99" s="49">
         <f>I99/H99</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N99" s="49">
         <f>J99/H99</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O99" s="49">
         <f>K99/H99</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P99" s="49">
         <f>L99/H99</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q99" s="29" t="inlineStr">
         <is>
@@ -4624,19 +4643,19 @@
       </c>
       <c r="M100" s="52">
         <f>I100/H100</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N100" s="52">
         <f>J100/H100</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O100" s="52">
         <f>K100/H100</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P100" s="52">
         <f>L100/H100</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q100" s="30" t="inlineStr">
         <is>
@@ -4690,19 +4709,19 @@
       </c>
       <c r="M101" s="49">
         <f>I101/H101</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N101" s="49">
         <f>J101/H101</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O101" s="49">
         <f>K101/H101</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P101" s="49">
         <f>L101/H101</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q101" s="29" t="inlineStr">
         <is>
@@ -4756,19 +4775,19 @@
       </c>
       <c r="M102" s="52">
         <f>I102/H102</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N102" s="52">
         <f>J102/H102</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O102" s="52">
         <f>K102/H102</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P102" s="52">
         <f>L102/H102</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q102" s="30" t="inlineStr">
         <is>
@@ -4822,19 +4841,19 @@
       </c>
       <c r="M103" s="49">
         <f>I103/H103</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N103" s="49">
         <f>J103/H103</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O103" s="49">
         <f>K103/H103</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P103" s="49">
         <f>L103/H103</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q103" s="29" t="inlineStr">
         <is>
@@ -4888,19 +4907,19 @@
       </c>
       <c r="M104" s="52">
         <f>I104/H104</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N104" s="52">
         <f>J104/H104</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O104" s="52">
         <f>K104/H104</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P104" s="52">
         <f>L104/H104</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q104" s="30" t="inlineStr">
         <is>
@@ -4954,19 +4973,19 @@
       </c>
       <c r="M105" s="49">
         <f>I105/H105</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N105" s="49">
         <f>J105/H105</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O105" s="49">
         <f>K105/H105</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P105" s="49">
         <f>L105/H105</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q105" s="29" t="inlineStr">
         <is>
@@ -5020,19 +5039,19 @@
       </c>
       <c r="M106" s="52">
         <f>I106/H106</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N106" s="52">
         <f>J106/H106</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O106" s="52">
         <f>K106/H106</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P106" s="52">
         <f>L106/H106</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q106" s="30" t="inlineStr">
         <is>
@@ -5086,19 +5105,19 @@
       </c>
       <c r="M107" s="49">
         <f>I107/H107</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N107" s="49">
         <f>J107/H107</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O107" s="49">
         <f>K107/H107</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P107" s="49">
         <f>L107/H107</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q107" s="29" t="inlineStr">
         <is>
@@ -5152,19 +5171,19 @@
       </c>
       <c r="M108" s="52">
         <f>I108/H108</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N108" s="52">
         <f>J108/H108</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O108" s="52">
         <f>K108/H108</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P108" s="52">
         <f>L108/H108</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q108" s="30" t="inlineStr">
         <is>
@@ -5218,19 +5237,19 @@
       </c>
       <c r="M109" s="49">
         <f>I109/H109</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N109" s="49">
         <f>J109/H109</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O109" s="49">
         <f>K109/H109</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P109" s="49">
         <f>L109/H109</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q109" s="29" t="inlineStr">
         <is>
@@ -5284,19 +5303,19 @@
       </c>
       <c r="M110" s="52">
         <f>I110/H110</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N110" s="52">
         <f>J110/H110</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O110" s="52">
         <f>K110/H110</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P110" s="52">
         <f>L110/H110</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q110" s="30" t="inlineStr">
         <is>
@@ -5350,19 +5369,19 @@
       </c>
       <c r="M111" s="49">
         <f>I111/H111</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N111" s="49">
         <f>J111/H111</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O111" s="49">
         <f>K111/H111</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P111" s="49">
         <f>L111/H111</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q111" s="29" t="inlineStr">
         <is>
@@ -5416,19 +5435,19 @@
       </c>
       <c r="M112" s="52">
         <f>I112/H112</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N112" s="52">
         <f>J112/H112</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O112" s="52">
         <f>K112/H112</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P112" s="52">
         <f>L112/H112</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q112" s="30" t="inlineStr">
         <is>
@@ -5482,19 +5501,19 @@
       </c>
       <c r="M113" s="49">
         <f>I113/H113</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N113" s="49">
         <f>J113/H113</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O113" s="49">
         <f>K113/H113</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P113" s="49">
         <f>L113/H113</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q113" s="29" t="inlineStr">
         <is>
@@ -5548,19 +5567,19 @@
       </c>
       <c r="M114" s="52">
         <f>I114/H114</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N114" s="52">
         <f>J114/H114</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O114" s="52">
         <f>K114/H114</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P114" s="52">
         <f>L114/H114</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q114" s="30" t="inlineStr">
         <is>
@@ -5614,19 +5633,19 @@
       </c>
       <c r="M115" s="49">
         <f>I115/H115</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N115" s="49">
         <f>J115/H115</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O115" s="49">
         <f>K115/H115</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P115" s="49">
         <f>L115/H115</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q115" s="29" t="inlineStr">
         <is>
@@ -5680,19 +5699,19 @@
       </c>
       <c r="M116" s="52">
         <f>I116/H116</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N116" s="52">
         <f>J116/H116</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O116" s="52">
         <f>K116/H116</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P116" s="52">
         <f>L116/H116</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q116" s="30" t="inlineStr">
         <is>
@@ -5746,19 +5765,19 @@
       </c>
       <c r="M117" s="49">
         <f>I117/H117</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N117" s="49">
         <f>J117/H117</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O117" s="49">
         <f>K117/H117</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P117" s="49">
         <f>L117/H117</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q117" s="29" t="inlineStr">
         <is>
@@ -5812,19 +5831,19 @@
       </c>
       <c r="M118" s="52">
         <f>I118/H118</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N118" s="52">
         <f>J118/H118</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O118" s="52">
         <f>K118/H118</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P118" s="52">
         <f>L118/H118</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q118" s="30" t="inlineStr">
         <is>
@@ -5878,19 +5897,19 @@
       </c>
       <c r="M119" s="49">
         <f>I119/H119</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N119" s="49">
         <f>J119/H119</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O119" s="49">
         <f>K119/H119</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P119" s="49">
         <f>L119/H119</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q119" s="29" t="inlineStr">
         <is>
@@ -5944,19 +5963,19 @@
       </c>
       <c r="M120" s="52">
         <f>I120/H120</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N120" s="52">
         <f>J120/H120</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O120" s="52">
         <f>K120/H120</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P120" s="52">
         <f>L120/H120</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q120" s="30" t="inlineStr">
         <is>
@@ -6010,19 +6029,19 @@
       </c>
       <c r="M121" s="49">
         <f>I121/H121</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N121" s="49">
         <f>J121/H121</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O121" s="49">
         <f>K121/H121</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P121" s="49">
         <f>L121/H121</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q121" s="29" t="inlineStr">
         <is>
@@ -6076,19 +6095,19 @@
       </c>
       <c r="M122" s="52">
         <f>I122/H122</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N122" s="52">
         <f>J122/H122</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O122" s="52">
         <f>K122/H122</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P122" s="52">
         <f>L122/H122</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q122" s="30" t="inlineStr">
         <is>
@@ -6142,19 +6161,19 @@
       </c>
       <c r="M123" s="49">
         <f>I123/H123</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N123" s="49">
         <f>J123/H123</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O123" s="49">
         <f>K123/H123</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P123" s="49">
         <f>L123/H123</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q123" s="29" t="inlineStr">
         <is>
@@ -6208,19 +6227,19 @@
       </c>
       <c r="M124" s="52">
         <f>I124/H124</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N124" s="52">
         <f>J124/H124</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O124" s="52">
         <f>K124/H124</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P124" s="52">
         <f>L124/H124</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q124" s="30" t="inlineStr">
         <is>
@@ -6274,19 +6293,19 @@
       </c>
       <c r="M125" s="49">
         <f>I125/H125</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N125" s="49">
         <f>J125/H125</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O125" s="49">
         <f>K125/H125</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P125" s="49">
         <f>L125/H125</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q125" s="29" t="inlineStr">
         <is>
@@ -6340,19 +6359,19 @@
       </c>
       <c r="M126" s="52">
         <f>I126/H126</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N126" s="52">
         <f>J126/H126</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O126" s="52">
         <f>K126/H126</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P126" s="52">
         <f>L126/H126</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q126" s="30" t="inlineStr">
         <is>
@@ -6406,19 +6425,19 @@
       </c>
       <c r="M127" s="49">
         <f>I127/H127</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N127" s="49">
         <f>J127/H127</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O127" s="49">
         <f>K127/H127</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P127" s="49">
         <f>L127/H127</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q127" s="29" t="inlineStr">
         <is>
@@ -6472,19 +6491,19 @@
       </c>
       <c r="M128" s="52">
         <f>I128/H128</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N128" s="52">
         <f>J128/H128</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O128" s="52">
         <f>K128/H128</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P128" s="52">
         <f>L128/H128</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q128" s="30" t="inlineStr">
         <is>
@@ -6538,19 +6557,19 @@
       </c>
       <c r="M129" s="49">
         <f>I129/H129</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N129" s="49">
         <f>J129/H129</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O129" s="49">
         <f>K129/H129</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P129" s="49">
         <f>L129/H129</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q129" s="29" t="inlineStr">
         <is>
@@ -6604,19 +6623,19 @@
       </c>
       <c r="M130" s="52">
         <f>I130/H130</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N130" s="52">
         <f>J130/H130</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O130" s="52">
         <f>K130/H130</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P130" s="52">
         <f>L130/H130</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q130" s="30" t="inlineStr">
         <is>
@@ -6670,19 +6689,19 @@
       </c>
       <c r="M131" s="49">
         <f>I131/H131</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N131" s="49">
         <f>J131/H131</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O131" s="49">
         <f>K131/H131</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P131" s="49">
         <f>L131/H131</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q131" s="29" t="inlineStr">
         <is>
@@ -6736,19 +6755,19 @@
       </c>
       <c r="M132" s="52">
         <f>I132/H132</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N132" s="52">
         <f>J132/H132</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O132" s="52">
         <f>K132/H132</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P132" s="52">
         <f>L132/H132</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q132" s="30" t="inlineStr">
         <is>
@@ -6802,19 +6821,19 @@
       </c>
       <c r="M133" s="49">
         <f>I133/H133</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N133" s="49">
         <f>J133/H133</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O133" s="49">
         <f>K133/H133</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P133" s="49">
         <f>L133/H133</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q133" s="29" t="inlineStr">
         <is>
@@ -6868,19 +6887,19 @@
       </c>
       <c r="M134" s="52">
         <f>I134/H134</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N134" s="52">
         <f>J134/H134</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O134" s="52">
         <f>K134/H134</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P134" s="52">
         <f>L134/H134</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q134" s="30" t="inlineStr">
         <is>
@@ -6934,19 +6953,19 @@
       </c>
       <c r="M135" s="49">
         <f>I135/H135</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N135" s="49">
         <f>J135/H135</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O135" s="49">
         <f>K135/H135</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P135" s="49">
         <f>L135/H135</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q135" s="29" t="inlineStr">
         <is>
@@ -7000,19 +7019,19 @@
       </c>
       <c r="M136" s="52">
         <f>I136/H136</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N136" s="52">
         <f>J136/H136</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O136" s="52">
         <f>K136/H136</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P136" s="52">
         <f>L136/H136</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q136" s="30" t="inlineStr">
         <is>
@@ -7066,19 +7085,19 @@
       </c>
       <c r="M137" s="49">
         <f>I137/H137</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N137" s="49">
         <f>J137/H137</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O137" s="49">
         <f>K137/H137</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P137" s="49">
         <f>L137/H137</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q137" s="29" t="inlineStr">
         <is>
@@ -7132,19 +7151,19 @@
       </c>
       <c r="M138" s="52">
         <f>I138/H138</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N138" s="52">
         <f>J138/H138</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O138" s="52">
         <f>K138/H138</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P138" s="52">
         <f>L138/H138</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q138" s="30" t="inlineStr">
         <is>
@@ -7198,19 +7217,19 @@
       </c>
       <c r="M139" s="49">
         <f>I139/H139</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N139" s="49">
         <f>J139/H139</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O139" s="49">
         <f>K139/H139</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P139" s="49">
         <f>L139/H139</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q139" s="29" t="inlineStr">
         <is>
@@ -7264,19 +7283,19 @@
       </c>
       <c r="M140" s="52">
         <f>I140/H140</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N140" s="52">
         <f>J140/H140</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O140" s="52">
         <f>K140/H140</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P140" s="52">
         <f>L140/H140</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q140" s="30" t="inlineStr">
         <is>
@@ -7330,19 +7349,19 @@
       </c>
       <c r="M141" s="49">
         <f>I141/H141</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N141" s="49">
         <f>J141/H141</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O141" s="49">
         <f>K141/H141</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P141" s="49">
         <f>L141/H141</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q141" s="29" t="inlineStr">
         <is>
@@ -7396,19 +7415,19 @@
       </c>
       <c r="M142" s="52">
         <f>I142/H142</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N142" s="52">
         <f>J142/H142</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O142" s="52">
         <f>K142/H142</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P142" s="52">
         <f>L142/H142</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q142" s="30" t="inlineStr">
         <is>
@@ -7462,19 +7481,19 @@
       </c>
       <c r="M143" s="49">
         <f>I143/H143</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N143" s="49">
         <f>J143/H143</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O143" s="49">
         <f>K143/H143</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P143" s="49">
         <f>L143/H143</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q143" s="29" t="inlineStr">
         <is>
@@ -7528,19 +7547,19 @@
       </c>
       <c r="M144" s="52">
         <f>I144/H144</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N144" s="52">
         <f>J144/H144</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O144" s="52">
         <f>K144/H144</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P144" s="52">
         <f>L144/H144</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q144" s="30" t="inlineStr">
         <is>
@@ -7594,19 +7613,19 @@
       </c>
       <c r="M145" s="49">
         <f>I145/H145</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N145" s="49">
         <f>J145/H145</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O145" s="49">
         <f>K145/H145</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P145" s="49">
         <f>L145/H145</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q145" s="29" t="inlineStr">
         <is>
@@ -7660,19 +7679,19 @@
       </c>
       <c r="M146" s="52">
         <f>I146/H146</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N146" s="52">
         <f>J146/H146</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O146" s="52">
         <f>K146/H146</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P146" s="52">
         <f>L146/H146</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q146" s="30" t="inlineStr">
         <is>
@@ -7726,19 +7745,19 @@
       </c>
       <c r="M147" s="49">
         <f>I147/H147</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N147" s="49">
         <f>J147/H147</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O147" s="49">
         <f>K147/H147</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P147" s="49">
         <f>L147/H147</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q147" s="29" t="inlineStr">
         <is>
@@ -7792,19 +7811,19 @@
       </c>
       <c r="M148" s="52">
         <f>I148/H148</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N148" s="52">
         <f>J148/H148</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O148" s="52">
         <f>K148/H148</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P148" s="52">
         <f>L148/H148</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q148" s="30" t="inlineStr">
         <is>
@@ -7858,19 +7877,19 @@
       </c>
       <c r="M149" s="49">
         <f>I149/H149</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N149" s="49">
         <f>J149/H149</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O149" s="49">
         <f>K149/H149</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P149" s="49">
         <f>L149/H149</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q149" s="29" t="inlineStr">
         <is>
@@ -7924,19 +7943,19 @@
       </c>
       <c r="M150" s="52">
         <f>I150/H150</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N150" s="52">
         <f>J150/H150</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O150" s="52">
         <f>K150/H150</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P150" s="52">
         <f>L150/H150</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q150" s="30" t="inlineStr">
         <is>
@@ -7990,19 +8009,19 @@
       </c>
       <c r="M151" s="49">
         <f>I151/H151</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N151" s="49">
         <f>J151/H151</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O151" s="49">
         <f>K151/H151</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P151" s="49">
         <f>L151/H151</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q151" s="29" t="inlineStr">
         <is>
@@ -8056,19 +8075,19 @@
       </c>
       <c r="M152" s="52">
         <f>I152/H152</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N152" s="52">
         <f>J152/H152</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O152" s="52">
         <f>K152/H152</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P152" s="52">
         <f>L152/H152</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q152" s="30" t="inlineStr">
         <is>
@@ -8122,19 +8141,19 @@
       </c>
       <c r="M153" s="49">
         <f>I153/H153</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N153" s="49">
         <f>J153/H153</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O153" s="49">
         <f>K153/H153</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P153" s="49">
         <f>L153/H153</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q153" s="29" t="inlineStr">
         <is>
@@ -8188,19 +8207,19 @@
       </c>
       <c r="M154" s="52">
         <f>I154/H154</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N154" s="52">
         <f>J154/H154</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O154" s="52">
         <f>K154/H154</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P154" s="52">
         <f>L154/H154</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q154" s="30" t="inlineStr">
         <is>
@@ -8254,19 +8273,19 @@
       </c>
       <c r="M155" s="49">
         <f>I155/H155</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N155" s="49">
         <f>J155/H155</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O155" s="49">
         <f>K155/H155</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P155" s="49">
         <f>L155/H155</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q155" s="29" t="inlineStr">
         <is>
@@ -8320,19 +8339,19 @@
       </c>
       <c r="M156" s="52">
         <f>I156/H156</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N156" s="52">
         <f>J156/H156</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O156" s="52">
         <f>K156/H156</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P156" s="52">
         <f>L156/H156</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q156" s="30" t="inlineStr">
         <is>
@@ -8386,19 +8405,19 @@
       </c>
       <c r="M157" s="49">
         <f>I157/H157</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N157" s="49">
         <f>J157/H157</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O157" s="49">
         <f>K157/H157</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P157" s="49">
         <f>L157/H157</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q157" s="29" t="inlineStr">
         <is>
@@ -8452,19 +8471,19 @@
       </c>
       <c r="M158" s="52">
         <f>I158/H158</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N158" s="52">
         <f>J158/H158</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O158" s="52">
         <f>K158/H158</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P158" s="52">
         <f>L158/H158</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q158" s="30" t="inlineStr">
         <is>
@@ -8518,19 +8537,19 @@
       </c>
       <c r="M159" s="49">
         <f>I159/H159</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N159" s="49">
         <f>J159/H159</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O159" s="49">
         <f>K159/H159</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P159" s="49">
         <f>L159/H159</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q159" s="29" t="inlineStr">
         <is>
@@ -8584,19 +8603,19 @@
       </c>
       <c r="M160" s="52">
         <f>I160/H160</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N160" s="52">
         <f>J160/H160</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O160" s="52">
         <f>K160/H160</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P160" s="52">
         <f>L160/H160</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q160" s="30" t="inlineStr">
         <is>
@@ -8650,19 +8669,19 @@
       </c>
       <c r="M161" s="49">
         <f>I161/H161</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N161" s="49">
         <f>J161/H161</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O161" s="49">
         <f>K161/H161</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P161" s="49">
         <f>L161/H161</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q161" s="29" t="inlineStr">
         <is>
@@ -8716,19 +8735,19 @@
       </c>
       <c r="M162" s="52">
         <f>I162/H162</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N162" s="52">
         <f>J162/H162</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O162" s="52">
         <f>K162/H162</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P162" s="52">
         <f>L162/H162</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q162" s="30" t="inlineStr">
         <is>
@@ -8782,19 +8801,19 @@
       </c>
       <c r="M163" s="49">
         <f>I163/H163</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N163" s="49">
         <f>J163/H163</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O163" s="49">
         <f>K163/H163</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P163" s="49">
         <f>L163/H163</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q163" s="29" t="inlineStr">
         <is>
@@ -8848,19 +8867,19 @@
       </c>
       <c r="M164" s="52">
         <f>I164/H164</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N164" s="52">
         <f>J164/H164</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O164" s="52">
         <f>K164/H164</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P164" s="52">
         <f>L164/H164</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q164" s="30" t="inlineStr">
         <is>
@@ -8914,19 +8933,19 @@
       </c>
       <c r="M165" s="49">
         <f>I165/H165</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N165" s="49">
         <f>J165/H165</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O165" s="49">
         <f>K165/H165</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P165" s="49">
         <f>L165/H165</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q165" s="29" t="inlineStr">
         <is>
@@ -8980,19 +8999,19 @@
       </c>
       <c r="M166" s="52">
         <f>I166/H166</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N166" s="52">
         <f>J166/H166</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O166" s="52">
         <f>K166/H166</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P166" s="52">
         <f>L166/H166</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q166" s="30" t="inlineStr">
         <is>
@@ -9046,19 +9065,19 @@
       </c>
       <c r="M167" s="49">
         <f>I167/H167</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N167" s="49">
         <f>J167/H167</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O167" s="49">
         <f>K167/H167</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P167" s="49">
         <f>L167/H167</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q167" s="29" t="inlineStr">
         <is>
@@ -9112,19 +9131,19 @@
       </c>
       <c r="M168" s="52">
         <f>I168/H168</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N168" s="52">
         <f>J168/H168</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O168" s="52">
         <f>K168/H168</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P168" s="52">
         <f>L168/H168</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q168" s="30" t="inlineStr">
         <is>
@@ -9178,19 +9197,19 @@
       </c>
       <c r="M169" s="49">
         <f>I169/H169</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N169" s="49">
         <f>J169/H169</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O169" s="49">
         <f>K169/H169</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P169" s="49">
         <f>L169/H169</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q169" s="29" t="inlineStr">
         <is>
@@ -9244,19 +9263,19 @@
       </c>
       <c r="M170" s="52">
         <f>I170/H170</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N170" s="52">
         <f>J170/H170</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O170" s="52">
         <f>K170/H170</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P170" s="52">
         <f>L170/H170</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q170" s="30" t="inlineStr">
         <is>
@@ -9310,19 +9329,19 @@
       </c>
       <c r="M171" s="49">
         <f>I171/H171</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N171" s="49">
         <f>J171/H171</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O171" s="49">
         <f>K171/H171</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P171" s="49">
         <f>L171/H171</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q171" s="29" t="inlineStr">
         <is>
@@ -9376,19 +9395,19 @@
       </c>
       <c r="M172" s="52">
         <f>I172/H172</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N172" s="52">
         <f>J172/H172</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O172" s="52">
         <f>K172/H172</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P172" s="52">
         <f>L172/H172</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q172" s="30" t="inlineStr">
         <is>
@@ -9442,19 +9461,19 @@
       </c>
       <c r="M173" s="49">
         <f>I173/H173</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N173" s="49">
         <f>J173/H173</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O173" s="49">
         <f>K173/H173</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P173" s="49">
         <f>L173/H173</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q173" s="29" t="inlineStr">
         <is>
@@ -9508,19 +9527,19 @@
       </c>
       <c r="M174" s="52">
         <f>I174/H174</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N174" s="52">
         <f>J174/H174</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O174" s="52">
         <f>K174/H174</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P174" s="52">
         <f>L174/H174</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q174" s="30" t="inlineStr">
         <is>
@@ -9574,19 +9593,19 @@
       </c>
       <c r="M175" s="49">
         <f>I175/H175</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N175" s="49">
         <f>J175/H175</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O175" s="49">
         <f>K175/H175</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P175" s="49">
         <f>L175/H175</f>
-        <v/>
+        <v>0.65</v>
       </c>
       <c r="Q175" s="29" t="inlineStr">
         <is>
@@ -9640,19 +9659,19 @@
       </c>
       <c r="M176" s="52">
         <f>I176/H176</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N176" s="52">
         <f>J176/H176</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O176" s="52">
         <f>K176/H176</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P176" s="52">
         <f>L176/H176</f>
-        <v/>
+        <v>0.7</v>
       </c>
       <c r="Q176" s="30" t="inlineStr">
         <is>
@@ -9706,19 +9725,19 @@
       </c>
       <c r="M177" s="49">
         <f>I177/H177</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N177" s="49">
         <f>J177/H177</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O177" s="49">
         <f>K177/H177</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P177" s="49">
         <f>L177/H177</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q177" s="29" t="inlineStr">
         <is>
@@ -9772,19 +9791,19 @@
       </c>
       <c r="M178" s="52">
         <f>I178/H178</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N178" s="52">
         <f>J178/H178</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O178" s="52">
         <f>K178/H178</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P178" s="52">
         <f>L178/H178</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="Q178" s="30" t="inlineStr">
         <is>
@@ -9838,19 +9857,19 @@
       </c>
       <c r="M179" s="49">
         <f>I179/H179</f>
-        <v/>
+        <v>0.45</v>
       </c>
       <c r="N179" s="49">
         <f>J179/H179</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O179" s="49">
         <f>K179/H179</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P179" s="49">
         <f>L179/H179</f>
-        <v/>
+        <v>0.5</v>
       </c>
       <c r="Q179" s="29" t="inlineStr">
         <is>
@@ -9904,19 +9923,19 @@
       </c>
       <c r="M180" s="52">
         <f>I180/H180</f>
-        <v/>
+        <v>0.3</v>
       </c>
       <c r="N180" s="52">
         <f>J180/H180</f>
-        <v/>
+        <v>0.3</v>
       </c>
       <c r="O180" s="52">
         <f>K180/H180</f>
-        <v/>
+        <v>0.2</v>
       </c>
       <c r="P180" s="52">
         <f>L180/H180</f>
-        <v/>
+        <v>0.7</v>
       </c>
       <c r="Q180" s="30" t="inlineStr">
         <is>
@@ -9970,19 +9989,19 @@
       </c>
       <c r="M181" s="49">
         <f>I181/H181</f>
-        <v/>
+        <v>0.1</v>
       </c>
       <c r="N181" s="49">
         <f>J181/H181</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O181" s="49">
         <f>K181/H181</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P181" s="49">
         <f>L181/H181</f>
-        <v/>
+        <v>0.7</v>
       </c>
       <c r="Q181" s="29" t="inlineStr">
         <is>
@@ -10036,19 +10055,19 @@
       </c>
       <c r="M182" s="52">
         <f>I182/H182</f>
-        <v/>
+        <v>0.15</v>
       </c>
       <c r="N182" s="52">
         <f>J182/H182</f>
-        <v/>
+        <v>0.15</v>
       </c>
       <c r="O182" s="52">
         <f>K182/H182</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P182" s="52">
         <f>L182/H182</f>
-        <v/>
+        <v>0.9</v>
       </c>
       <c r="Q182" s="30" t="inlineStr">
         <is>
@@ -10102,19 +10121,19 @@
       </c>
       <c r="M183" s="49">
         <f>I183/H183</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N183" s="49">
         <f>J183/H183</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O183" s="49">
         <f>K183/H183</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P183" s="49">
         <f>L183/H183</f>
-        <v/>
+        <v>0.95</v>
       </c>
       <c r="Q183" s="29" t="inlineStr">
         <is>
@@ -10168,19 +10187,19 @@
       </c>
       <c r="M184" s="52">
         <f>I184/H184</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="N184" s="52">
         <f>J184/H184</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O184" s="52">
         <f>K184/H184</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P184" s="52">
         <f>L184/H184</f>
-        <v/>
+        <v>0.95</v>
       </c>
       <c r="Q184" s="30" t="inlineStr">
         <is>
@@ -10234,19 +10253,19 @@
       </c>
       <c r="M185" s="49">
         <f>I185/H185</f>
-        <v/>
+        <v>0.35</v>
       </c>
       <c r="N185" s="49">
         <f>J185/H185</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O185" s="49">
         <f>K185/H185</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="P185" s="49">
         <f>L185/H185</f>
-        <v/>
+        <v>0.65</v>
       </c>
       <c r="Q185" s="29" t="inlineStr">
         <is>
@@ -10300,19 +10319,19 @@
       </c>
       <c r="M186" s="52">
         <f>I186/H186</f>
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="N186" s="52">
         <f>J186/H186</f>
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="O186" s="52">
         <f>K186/H186</f>
-        <v/>
+        <v>0.4</v>
       </c>
       <c r="P186" s="52">
         <f>L186/H186</f>
-        <v/>
+        <v>0.55</v>
       </c>
       <c r="Q186" s="30" t="inlineStr">
         <is>
@@ -10339,7 +10358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N237"/>
+  <dimension ref="A1:N237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" style="25" min="1" max="1"/>
@@ -10358,6 +10377,7 @@
     <col width="27" customWidth="1" style="25" min="15" max="15"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="26" customHeight="1" s="25">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -10387,6 +10407,7 @@
       <c r="M4" s="3" t="n"/>
       <c r="N4" s="3" t="n"/>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
@@ -10394,6 +10415,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="34" customHeight="1" s="25">
       <c r="B8" s="11" t="inlineStr">
         <is>
@@ -10488,7 +10510,7 @@
       </c>
       <c r="K9" s="49">
         <f>J9/D9</f>
-        <v/>
+        <v>0.8833333333333333</v>
       </c>
       <c r="L9" s="48" t="n">
         <v>0</v>
@@ -10531,7 +10553,7 @@
       </c>
       <c r="K10" s="52">
         <f>J10/D10</f>
-        <v/>
+        <v>0.9666666666666667</v>
       </c>
       <c r="L10" s="51" t="n">
         <v>0</v>
@@ -10574,7 +10596,7 @@
       </c>
       <c r="K11" s="49">
         <f>J11/D11</f>
-        <v/>
+        <v>0.8333333333333334</v>
       </c>
       <c r="L11" s="48" t="n">
         <v>0</v>
@@ -10617,7 +10639,7 @@
       </c>
       <c r="K12" s="52">
         <f>J12/D12</f>
-        <v/>
+        <v>0.8</v>
       </c>
       <c r="L12" s="51" t="n">
         <v>0</v>
@@ -10660,7 +10682,7 @@
       </c>
       <c r="K13" s="49">
         <f>J13/D13</f>
-        <v/>
+        <v>0.8333333333333334</v>
       </c>
       <c r="L13" s="48" t="n">
         <v>0</v>
@@ -10672,6 +10694,7 @@
       </c>
     </row>
     <row r="14" ht="23" customHeight="1" s="25"/>
+    <row r="15"/>
     <row r="16" ht="19" customHeight="1" s="25">
       <c r="B16" s="24" t="inlineStr">
         <is>
@@ -10700,6 +10723,8 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
+    <row r="21"/>
     <row r="22" ht="22" customHeight="1" s="25">
       <c r="B22" s="37" t="inlineStr">
         <is>
@@ -10718,6 +10743,7 @@
       <c r="L22" s="37" t="n"/>
       <c r="M22" s="37" t="n"/>
     </row>
+    <row r="23"/>
     <row r="24" ht="44" customHeight="1" s="25">
       <c r="B24" s="45" t="inlineStr">
         <is>
@@ -11770,6 +11796,7 @@
         </is>
       </c>
     </row>
+    <row r="65"/>
     <row r="66">
       <c r="B66" t="inlineStr">
         <is>
@@ -11777,6 +11804,8 @@
         </is>
       </c>
     </row>
+    <row r="67"/>
+    <row r="68"/>
     <row r="69" ht="34" customHeight="1" s="25"/>
     <row r="70" ht="23" customHeight="1" s="25"/>
     <row r="71" ht="22" customHeight="1" s="25">
@@ -15905,6 +15934,11 @@
         </is>
       </c>
     </row>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
     <row r="195" ht="22" customHeight="1" s="25">
       <c r="B195" s="37" t="inlineStr">
         <is>
@@ -15923,6 +15957,7 @@
       <c r="L195" s="37" t="n"/>
       <c r="M195" s="37" t="n"/>
     </row>
+    <row r="196"/>
     <row r="197" ht="44" customHeight="1" s="25">
       <c r="B197" s="45" t="inlineStr">
         <is>
@@ -16110,6 +16145,7 @@
         </is>
       </c>
     </row>
+    <row r="202"/>
     <row r="203">
       <c r="B203" t="inlineStr">
         <is>
@@ -16117,6 +16153,8 @@
         </is>
       </c>
     </row>
+    <row r="204"/>
+    <row r="205"/>
     <row r="206" ht="22" customHeight="1" s="25">
       <c r="B206" s="37" t="inlineStr">
         <is>
@@ -16135,6 +16173,7 @@
       <c r="L206" s="37" t="n"/>
       <c r="M206" s="37" t="n"/>
     </row>
+    <row r="207"/>
     <row r="208">
       <c r="B208" s="11" t="inlineStr">
         <is>
@@ -16849,7 +16888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N64"/>
+  <dimension ref="A1:N64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" style="25" min="1" max="1"/>
@@ -16864,6 +16903,7 @@
     <col width="10" customWidth="1" style="25" min="10" max="10"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="26" customHeight="1" s="25">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -16893,6 +16933,7 @@
       <c r="M4" s="3" t="n"/>
       <c r="N4" s="3" t="n"/>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
@@ -16900,6 +16941,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="34" customHeight="1" s="25">
       <c r="B8" s="11" t="inlineStr">
         <is>
@@ -17530,6 +17572,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="19" customHeight="1" s="25">
       <c r="B24" s="24" t="inlineStr">
         <is>
@@ -17551,6 +17594,8 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
+    <row r="28"/>
     <row r="29">
       <c r="B29" s="4" t="inlineStr">
         <is>
@@ -17558,6 +17603,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31" ht="34" customHeight="1" s="25">
       <c r="B31" s="11" t="inlineStr">
         <is>
@@ -17782,6 +17828,7 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39" ht="19" customHeight="1" s="25">
       <c r="B39" s="24" t="inlineStr">
         <is>
@@ -17789,6 +17836,8 @@
         </is>
       </c>
     </row>
+    <row r="40"/>
+    <row r="41"/>
     <row r="42">
       <c r="B42" s="4" t="inlineStr">
         <is>
@@ -17796,6 +17845,7 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44" ht="34" customHeight="1" s="25">
       <c r="B44" s="11" t="inlineStr">
         <is>
@@ -18018,6 +18068,7 @@
         </is>
       </c>
     </row>
+    <row r="50"/>
     <row r="51" ht="19" customHeight="1" s="25">
       <c r="B51" s="24" t="inlineStr">
         <is>
@@ -18039,6 +18090,8 @@
         </is>
       </c>
     </row>
+    <row r="54"/>
+    <row r="55"/>
     <row r="56">
       <c r="B56" s="4" t="inlineStr">
         <is>
@@ -18046,6 +18099,7 @@
         </is>
       </c>
     </row>
+    <row r="57"/>
     <row r="58" ht="34" customHeight="1" s="25">
       <c r="B58" s="11" t="inlineStr">
         <is>
@@ -18192,6 +18246,7 @@
         </is>
       </c>
     </row>
+    <row r="62"/>
     <row r="63" ht="19" customHeight="1" s="25">
       <c r="B63" s="24" t="inlineStr">
         <is>
@@ -18224,7 +18279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N67"/>
+  <dimension ref="A1:N67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" style="25" min="1" max="1"/>
@@ -18233,6 +18288,7 @@
     <col width="74" customWidth="1" style="25" min="4" max="4"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="26" customHeight="1" s="25">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -18262,6 +18318,7 @@
       <c r="M4" s="3" t="n"/>
       <c r="N4" s="3" t="n"/>
     </row>
+    <row r="5"/>
     <row r="6" ht="34" customHeight="1" s="25">
       <c r="B6" s="35" t="inlineStr">
         <is>
@@ -18370,6 +18427,8 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
+    <row r="16"/>
     <row r="17">
       <c r="B17" s="4" t="inlineStr">
         <is>
@@ -18440,6 +18499,8 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
+    <row r="28"/>
     <row r="29">
       <c r="B29" s="4" t="inlineStr">
         <is>
@@ -18447,6 +18508,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="B31" s="34" t="inlineStr">
         <is>
@@ -18495,6 +18557,8 @@
         </is>
       </c>
     </row>
+    <row r="35"/>
+    <row r="36"/>
     <row r="37">
       <c r="B37" s="4" t="inlineStr">
         <is>
@@ -18502,6 +18566,7 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39" ht="35" customHeight="1" s="25">
       <c r="B39" s="35" t="inlineStr">
         <is>
@@ -18944,6 +19009,7 @@
         </is>
       </c>
     </row>
+    <row r="65"/>
     <row r="66">
       <c r="B66" s="24" t="inlineStr">
         <is>

</xml_diff>